<commit_message>
feat(data): connect real Dien Bien comparison fields
</commit_message>
<xml_diff>
--- a/frontend/dataset/weather/data.xlsx
+++ b/frontend/dataset/weather/data.xlsx
@@ -521,17 +521,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>27.4</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>23.1</t>
+          <t>23.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>5.7</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -541,12 +541,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>8.6</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>25.6</t>
+          <t>23.0</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -571,7 +571,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-18T20:17:47.892511+00:00</t>
+          <t>2026-07-19T00:59:31.590951+00:00</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -608,17 +608,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>26.2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>23.2</t>
+          <t>23.3</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>17.5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -628,12 +628,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>29.9</t>
+          <t>26.3</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-07-18T20:17:47.892511+00:00</t>
+          <t>2026-07-19T00:59:31.590951+00:00</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -695,32 +695,32 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>30.6</t>
+          <t>30.8</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>22.4</t>
+          <t>22.2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>75</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>22.7</t>
+          <t>21.2</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-07-18T20:17:47.892511+00:00</t>
+          <t>2026-07-19T00:59:31.590951+00:00</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>31.4</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -792,22 +792,22 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>73</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>6.6</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>20.9</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-07-18T20:17:47.892511+00:00</t>
+          <t>2026-07-19T00:59:31.590951+00:00</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -869,32 +869,32 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>29.9</t>
+          <t>28.8</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>22.8</t>
+          <t>22.2</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>84</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>7.6</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>21.6</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-07-18T20:17:47.892511+00:00</t>
+          <t>2026-07-19T00:59:31.590951+00:00</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>27.9</t>
+          <t>28.7</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -966,22 +966,22 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>14.1</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>98</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>8.8</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>19.1</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-07-18T20:17:47.892511+00:00</t>
+          <t>2026-07-19T00:59:31.590951+00:00</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-07-18T20:17:47.892511+00:00</t>
+          <t>2026-07-19T00:59:31.590951+00:00</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">

</xml_diff>

<commit_message>
feat(data): connect real Dien Bien comparison fields (#55)
</commit_message>
<xml_diff>
--- a/frontend/dataset/weather/data.xlsx
+++ b/frontend/dataset/weather/data.xlsx
@@ -521,17 +521,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>27.4</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>23.1</t>
+          <t>23.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>5.7</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -541,12 +541,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>8.6</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>25.6</t>
+          <t>23.0</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -571,7 +571,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-18T20:17:47.892511+00:00</t>
+          <t>2026-07-19T00:59:31.590951+00:00</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -608,17 +608,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>26.2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>23.2</t>
+          <t>23.3</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>17.5</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -628,12 +628,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>29.9</t>
+          <t>26.3</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-07-18T20:17:47.892511+00:00</t>
+          <t>2026-07-19T00:59:31.590951+00:00</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -695,32 +695,32 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>30.6</t>
+          <t>30.8</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>22.4</t>
+          <t>22.2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>75</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>22.7</t>
+          <t>21.2</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-07-18T20:17:47.892511+00:00</t>
+          <t>2026-07-19T00:59:31.590951+00:00</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>31.4</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -792,22 +792,22 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>73</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>6.6</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>20.9</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-07-18T20:17:47.892511+00:00</t>
+          <t>2026-07-19T00:59:31.590951+00:00</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -869,32 +869,32 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>29.9</t>
+          <t>28.8</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>22.8</t>
+          <t>22.2</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>84</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>7.6</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>21.6</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-07-18T20:17:47.892511+00:00</t>
+          <t>2026-07-19T00:59:31.590951+00:00</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>27.9</t>
+          <t>28.7</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -966,22 +966,22 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>14.1</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>98</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>8.8</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>19.1</t>
+          <t>23.8</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-07-18T20:17:47.892511+00:00</t>
+          <t>2026-07-19T00:59:31.590951+00:00</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-07-18T20:17:47.892511+00:00</t>
+          <t>2026-07-19T00:59:31.590951+00:00</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">

</xml_diff>